<commit_message>
Small change to pOXA48 rep1
</commit_message>
<xml_diff>
--- a/data/pOXA48/rep1/Plate reader summary .xlsx
+++ b/data/pOXA48/rep1/Plate reader summary .xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11018"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vuhien/Desktop/labevolution exp/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/storage/hien/Hien PhD project new/Result/Full lab evolution exp/pOXA48 plasmid/20251106 1st rep/Plate reader/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12426994-6671-6D43-8F85-46ABF70B5F59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{005AE106-744E-FE42-B087-D4FB540E3F95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28500" yWindow="3440" windowWidth="28040" windowHeight="17440" xr2:uid="{3FAC46DD-0ED8-864C-AF4A-2C63C1C1825D}"/>
+    <workbookView xWindow="-17680" yWindow="6960" windowWidth="28040" windowHeight="17440" activeTab="2" xr2:uid="{3FAC46DD-0ED8-864C-AF4A-2C63C1C1825D}"/>
   </bookViews>
   <sheets>
     <sheet name="523-620" sheetId="1" r:id="rId1"/>
@@ -87,20 +87,20 @@
     <t>136h</t>
   </si>
   <si>
-    <t>150h</t>
+    <t>160h</t>
   </si>
   <si>
-    <t>174h</t>
+    <t>184h</t>
   </si>
   <si>
-    <t>198h</t>
+    <t>208h</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -125,13 +125,6 @@
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="18">
@@ -238,7 +231,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -307,46 +300,16 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
+      <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="thin">
+      <right style="medium">
         <color indexed="64"/>
       </right>
       <top style="thin">
         <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -385,7 +348,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -393,15 +356,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -435,37 +396,31 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="16" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="17" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="17" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -792,37 +747,37 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A1" s="6"/>
-      <c r="B1" s="6" t="s">
+      <c r="A1" s="5"/>
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="J1" s="5" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="1">
@@ -854,7 +809,7 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="5" t="s">
         <v>10</v>
       </c>
       <c r="B3" s="1">
@@ -886,7 +841,7 @@
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="5" t="s">
         <v>11</v>
       </c>
       <c r="B4" s="1">
@@ -918,7 +873,7 @@
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="5" t="s">
         <v>12</v>
       </c>
       <c r="B5" s="1">
@@ -950,7 +905,7 @@
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="5" t="s">
         <v>13</v>
       </c>
       <c r="B6" s="1">
@@ -982,7 +937,7 @@
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="5" t="s">
         <v>14</v>
       </c>
       <c r="B7" s="1">
@@ -1014,7 +969,7 @@
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="5" t="s">
         <v>15</v>
       </c>
       <c r="B8" s="1">
@@ -1046,104 +1001,104 @@
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A9" s="22" t="s">
+      <c r="A9" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="15">
+      <c r="B9" s="13">
         <v>14</v>
       </c>
-      <c r="C9" s="15">
+      <c r="C9" s="13">
         <v>428</v>
       </c>
-      <c r="D9" s="23">
+      <c r="D9" s="19">
         <v>7118</v>
       </c>
-      <c r="E9" s="17">
+      <c r="E9" s="15">
         <v>13208</v>
       </c>
-      <c r="F9" s="34">
+      <c r="F9" s="28">
         <v>6540</v>
       </c>
-      <c r="G9" s="16">
+      <c r="G9" s="14">
         <v>4882</v>
       </c>
-      <c r="H9" s="16">
+      <c r="H9" s="14">
         <v>4863</v>
       </c>
-      <c r="I9" s="16">
+      <c r="I9" s="14">
         <v>4937</v>
       </c>
-      <c r="J9" s="15">
+      <c r="J9" s="13">
         <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A10" s="22" t="s">
+      <c r="A10" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="15">
+      <c r="B10" s="13">
         <v>51</v>
       </c>
-      <c r="C10" s="15">
+      <c r="C10" s="13">
         <v>352</v>
       </c>
-      <c r="D10" s="16">
+      <c r="D10" s="14">
         <v>4923</v>
       </c>
-      <c r="E10" s="17">
+      <c r="E10" s="15">
         <v>12944</v>
       </c>
-      <c r="F10" s="35">
+      <c r="F10" s="29">
         <v>8430</v>
       </c>
-      <c r="G10" s="16">
+      <c r="G10" s="14">
         <v>4763</v>
       </c>
-      <c r="H10" s="16">
+      <c r="H10" s="14">
         <v>4907</v>
       </c>
-      <c r="I10" s="20">
+      <c r="I10" s="18">
         <v>4283</v>
       </c>
-      <c r="J10" s="15">
+      <c r="J10" s="13">
         <v>61</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A11" s="22" t="s">
+      <c r="A11" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="10">
+      <c r="B11" s="8">
         <v>66</v>
       </c>
-      <c r="C11" s="10">
+      <c r="C11" s="8">
         <v>240</v>
       </c>
-      <c r="D11" s="24">
+      <c r="D11" s="20">
         <v>4342</v>
       </c>
-      <c r="E11" s="11">
+      <c r="E11" s="9">
         <v>9387</v>
       </c>
-      <c r="F11" s="12">
+      <c r="F11" s="10">
         <v>6204</v>
       </c>
-      <c r="G11" s="24">
+      <c r="G11" s="20">
         <v>4444</v>
       </c>
-      <c r="H11" s="13">
+      <c r="H11" s="11">
         <v>3647</v>
       </c>
-      <c r="I11" s="14">
+      <c r="I11" s="12">
         <v>2525</v>
       </c>
-      <c r="J11" s="10">
+      <c r="J11" s="8">
         <v>54</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:J8">
-    <cfRule type="colorScale" priority="2">
+  <conditionalFormatting sqref="A1:J11">
+    <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -1152,8 +1107,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A1:J11">
-    <cfRule type="colorScale" priority="1">
+  <conditionalFormatting sqref="B2:J8">
+    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -1205,31 +1160,31 @@
       <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="7">
+      <c r="B2" s="6">
         <v>663</v>
       </c>
-      <c r="C2" s="7">
+      <c r="C2" s="6">
         <v>612</v>
       </c>
-      <c r="D2" s="7">
+      <c r="D2" s="6">
         <v>641</v>
       </c>
-      <c r="E2" s="7">
+      <c r="E2" s="6">
         <v>593</v>
       </c>
-      <c r="F2" s="7">
+      <c r="F2" s="6">
         <v>654</v>
       </c>
-      <c r="G2" s="7">
+      <c r="G2" s="6">
         <v>657</v>
       </c>
-      <c r="H2" s="7">
+      <c r="H2" s="6">
         <v>630</v>
       </c>
-      <c r="I2" s="7">
+      <c r="I2" s="6">
         <v>583</v>
       </c>
-      <c r="J2" s="8">
+      <c r="J2" s="7">
         <v>27</v>
       </c>
     </row>
@@ -1237,31 +1192,31 @@
       <c r="A3" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="7">
+      <c r="B3" s="6">
         <v>2355</v>
       </c>
-      <c r="C3" s="7">
+      <c r="C3" s="6">
         <v>2253</v>
       </c>
-      <c r="D3" s="7">
+      <c r="D3" s="6">
         <v>2238</v>
       </c>
-      <c r="E3" s="7">
+      <c r="E3" s="6">
         <v>2981</v>
       </c>
-      <c r="F3" s="7">
+      <c r="F3" s="6">
         <v>2655</v>
       </c>
-      <c r="G3" s="7">
+      <c r="G3" s="6">
         <v>2837</v>
       </c>
-      <c r="H3" s="7">
+      <c r="H3" s="6">
         <v>2405</v>
       </c>
-      <c r="I3" s="7">
+      <c r="I3" s="6">
         <v>2410</v>
       </c>
-      <c r="J3" s="8">
+      <c r="J3" s="7">
         <v>14</v>
       </c>
     </row>
@@ -1269,31 +1224,31 @@
       <c r="A4" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="7">
+      <c r="B4" s="6">
         <v>2663</v>
       </c>
-      <c r="C4" s="7">
+      <c r="C4" s="6">
         <v>889</v>
       </c>
-      <c r="D4" s="7">
+      <c r="D4" s="6">
         <v>2480</v>
       </c>
-      <c r="E4" s="7">
+      <c r="E4" s="6">
         <v>3984</v>
       </c>
-      <c r="F4" s="7">
+      <c r="F4" s="6">
         <v>3024</v>
       </c>
-      <c r="G4" s="7">
+      <c r="G4" s="6">
         <v>3044</v>
       </c>
-      <c r="H4" s="7">
+      <c r="H4" s="6">
         <v>2035</v>
       </c>
-      <c r="I4" s="7">
+      <c r="I4" s="6">
         <v>1931</v>
       </c>
-      <c r="J4" s="8">
+      <c r="J4" s="7">
         <v>19</v>
       </c>
     </row>
@@ -1301,31 +1256,31 @@
       <c r="A5" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="7">
+      <c r="B5" s="6">
         <v>19</v>
       </c>
-      <c r="C5" s="7">
+      <c r="C5" s="6">
         <v>687</v>
       </c>
-      <c r="D5" s="7">
+      <c r="D5" s="6">
         <v>4332</v>
       </c>
-      <c r="E5" s="7">
+      <c r="E5" s="6">
         <v>3248</v>
       </c>
-      <c r="F5" s="7">
+      <c r="F5" s="6">
         <v>4819</v>
       </c>
-      <c r="G5" s="7">
+      <c r="G5" s="6">
         <v>4340</v>
       </c>
-      <c r="H5" s="7">
+      <c r="H5" s="6">
         <v>4667</v>
       </c>
-      <c r="I5" s="7">
+      <c r="I5" s="6">
         <v>4689</v>
       </c>
-      <c r="J5" s="8">
+      <c r="J5" s="7">
         <v>25</v>
       </c>
     </row>
@@ -1333,31 +1288,31 @@
       <c r="A6" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="7">
+      <c r="B6" s="6">
         <v>25</v>
       </c>
-      <c r="C6" s="7">
+      <c r="C6" s="6">
         <v>517</v>
       </c>
-      <c r="D6" s="7">
+      <c r="D6" s="6">
         <v>5317</v>
       </c>
-      <c r="E6" s="7">
+      <c r="E6" s="6">
         <v>2759</v>
       </c>
-      <c r="F6" s="7">
+      <c r="F6" s="6">
         <v>5137</v>
       </c>
-      <c r="G6" s="7">
+      <c r="G6" s="6">
         <v>2626</v>
       </c>
-      <c r="H6" s="7">
+      <c r="H6" s="6">
         <v>4678</v>
       </c>
-      <c r="I6" s="7">
+      <c r="I6" s="6">
         <v>3513</v>
       </c>
-      <c r="J6" s="8">
+      <c r="J6" s="7">
         <v>27</v>
       </c>
     </row>
@@ -1365,31 +1320,31 @@
       <c r="A7" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="7">
+      <c r="B7" s="6">
         <v>28</v>
       </c>
-      <c r="C7" s="7">
+      <c r="C7" s="6">
         <v>345</v>
       </c>
-      <c r="D7" s="7">
+      <c r="D7" s="6">
         <v>3783</v>
       </c>
-      <c r="E7" s="7">
+      <c r="E7" s="6">
         <v>2252</v>
       </c>
-      <c r="F7" s="7">
+      <c r="F7" s="6">
         <v>4939</v>
       </c>
-      <c r="G7" s="7">
+      <c r="G7" s="6">
         <v>2797</v>
       </c>
-      <c r="H7" s="7">
+      <c r="H7" s="6">
         <v>3448</v>
       </c>
-      <c r="I7" s="7">
+      <c r="I7" s="6">
         <v>2802</v>
       </c>
-      <c r="J7" s="8">
+      <c r="J7" s="7">
         <v>22</v>
       </c>
     </row>
@@ -1397,133 +1352,133 @@
       <c r="A8" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="7">
+      <c r="B8" s="6">
         <v>24</v>
       </c>
-      <c r="C8" s="7">
+      <c r="C8" s="6">
         <v>219</v>
       </c>
-      <c r="D8" s="7">
+      <c r="D8" s="6">
         <v>3345</v>
       </c>
-      <c r="E8" s="7">
+      <c r="E8" s="6">
         <v>2229</v>
       </c>
-      <c r="F8" s="7">
+      <c r="F8" s="6">
         <v>6328</v>
       </c>
-      <c r="G8" s="7">
+      <c r="G8" s="6">
         <v>4132</v>
       </c>
-      <c r="H8" s="7">
+      <c r="H8" s="6">
         <v>2688</v>
       </c>
-      <c r="I8" s="7">
+      <c r="I8" s="6">
         <v>2763</v>
       </c>
-      <c r="J8" s="8">
+      <c r="J8" s="7">
         <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A9" s="25" t="s">
+      <c r="A9" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="15">
+      <c r="B9" s="13">
         <v>26</v>
       </c>
-      <c r="C9" s="15">
+      <c r="C9" s="13">
         <v>139</v>
       </c>
-      <c r="D9" s="23">
+      <c r="D9" s="19">
         <v>3474</v>
       </c>
-      <c r="E9" s="20">
+      <c r="E9" s="18">
         <v>2106</v>
       </c>
-      <c r="F9" s="17">
+      <c r="F9" s="15">
         <v>6287</v>
       </c>
-      <c r="G9" s="19">
+      <c r="G9" s="17">
         <v>4961</v>
       </c>
-      <c r="H9" s="16">
+      <c r="H9" s="14">
         <v>2430</v>
       </c>
-      <c r="I9" s="16">
+      <c r="I9" s="14">
         <v>2383</v>
       </c>
-      <c r="J9" s="26">
+      <c r="J9" s="21">
         <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A10" s="25" t="s">
+      <c r="A10" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="15">
+      <c r="B10" s="13">
         <v>39</v>
       </c>
-      <c r="C10" s="15">
+      <c r="C10" s="13">
         <v>77</v>
       </c>
-      <c r="D10" s="16">
+      <c r="D10" s="14">
         <v>2919</v>
       </c>
-      <c r="E10" s="16">
+      <c r="E10" s="14">
         <v>2711</v>
       </c>
-      <c r="F10" s="17">
+      <c r="F10" s="15">
         <v>7159</v>
       </c>
-      <c r="G10" s="18">
+      <c r="G10" s="16">
         <v>6162</v>
       </c>
-      <c r="H10" s="20">
+      <c r="H10" s="18">
         <v>2359</v>
       </c>
-      <c r="I10" s="20">
+      <c r="I10" s="18">
         <v>2074</v>
       </c>
-      <c r="J10" s="26">
+      <c r="J10" s="21">
         <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="27" t="s">
+      <c r="A11" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="28">
+      <c r="B11" s="22">
         <v>25</v>
       </c>
-      <c r="C11" s="28">
+      <c r="C11" s="22">
         <v>76</v>
       </c>
-      <c r="D11" s="29">
+      <c r="D11" s="23">
         <v>2486</v>
       </c>
-      <c r="E11" s="29">
+      <c r="E11" s="23">
         <v>2570</v>
       </c>
-      <c r="F11" s="30">
+      <c r="F11" s="24">
         <v>5717</v>
       </c>
-      <c r="G11" s="30">
+      <c r="G11" s="24">
         <v>5576</v>
       </c>
-      <c r="H11" s="31">
+      <c r="H11" s="25">
         <v>2015</v>
       </c>
-      <c r="I11" s="32">
+      <c r="I11" s="26">
         <v>1402</v>
       </c>
-      <c r="J11" s="33">
+      <c r="J11" s="27">
         <v>35</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
-  <conditionalFormatting sqref="B2:J8">
+  <conditionalFormatting sqref="A1:J1 B2:J11">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -1533,7 +1488,17 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A1:J11">
+  <conditionalFormatting sqref="B2:J8">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2:A11">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -1553,357 +1518,367 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A1" s="6"/>
-      <c r="B1" s="6" t="s">
+      <c r="A1" s="5"/>
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="J1" s="5" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="21">
+      <c r="B2" s="6">
         <v>0.17499999999999999</v>
       </c>
-      <c r="C2" s="21">
+      <c r="C2" s="6">
         <v>0.16600000000000001</v>
       </c>
-      <c r="D2" s="21">
+      <c r="D2" s="6">
         <v>0.17799999999999999</v>
       </c>
-      <c r="E2" s="21">
+      <c r="E2" s="6">
         <v>0.17100000000000001</v>
       </c>
-      <c r="F2" s="21">
+      <c r="F2" s="6">
         <v>0.191</v>
       </c>
-      <c r="G2" s="21">
+      <c r="G2" s="6">
         <v>0.19500000000000001</v>
       </c>
-      <c r="H2" s="21">
+      <c r="H2" s="6">
         <v>0.17699999999999999</v>
       </c>
-      <c r="I2" s="21">
+      <c r="I2" s="6">
         <v>0.17199999999999999</v>
       </c>
-      <c r="J2" s="21">
+      <c r="J2" s="6">
         <v>9.4E-2</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="21">
+      <c r="B3" s="6">
         <v>0.16600000000000001</v>
       </c>
-      <c r="C3" s="21">
+      <c r="C3" s="6">
         <v>0.13800000000000001</v>
       </c>
-      <c r="D3" s="21">
+      <c r="D3" s="6">
         <v>0.17</v>
       </c>
-      <c r="E3" s="21">
+      <c r="E3" s="6">
         <v>0.16900000000000001</v>
       </c>
-      <c r="F3" s="21">
+      <c r="F3" s="6">
         <v>0.19800000000000001</v>
       </c>
-      <c r="G3" s="21">
+      <c r="G3" s="6">
         <v>0.188</v>
       </c>
-      <c r="H3" s="21">
+      <c r="H3" s="6">
         <v>0.16700000000000001</v>
       </c>
-      <c r="I3" s="21">
+      <c r="I3" s="6">
         <v>0.16500000000000001</v>
       </c>
-      <c r="J3" s="21">
+      <c r="J3" s="6">
         <v>8.6999999999999994E-2</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="21">
+      <c r="B4" s="6">
         <v>0.16200000000000001</v>
       </c>
-      <c r="C4" s="21">
+      <c r="C4" s="6">
         <v>0.125</v>
       </c>
-      <c r="D4" s="21">
+      <c r="D4" s="6">
         <v>0.17299999999999999</v>
       </c>
-      <c r="E4" s="21">
+      <c r="E4" s="6">
         <v>0.249</v>
       </c>
-      <c r="F4" s="21">
+      <c r="F4" s="6">
         <v>0.20100000000000001</v>
       </c>
-      <c r="G4" s="21">
+      <c r="G4" s="6">
         <v>0.22500000000000001</v>
       </c>
-      <c r="H4" s="21">
+      <c r="H4" s="6">
         <v>0.17199999999999999</v>
       </c>
-      <c r="I4" s="21">
+      <c r="I4" s="6">
         <v>0.16600000000000001</v>
       </c>
-      <c r="J4" s="21">
+      <c r="J4" s="6">
         <v>0.09</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="21">
+      <c r="B5" s="6">
         <v>0.11899999999999999</v>
       </c>
-      <c r="C5" s="21">
+      <c r="C5" s="6">
         <v>0.11700000000000001</v>
       </c>
-      <c r="D5" s="21">
+      <c r="D5" s="6">
         <v>0.254</v>
       </c>
-      <c r="E5" s="21">
+      <c r="E5" s="6">
         <v>0.26100000000000001</v>
       </c>
-      <c r="F5" s="21">
+      <c r="F5" s="6">
         <v>0.314</v>
       </c>
-      <c r="G5" s="21">
+      <c r="G5" s="6">
         <v>0.27300000000000002</v>
       </c>
-      <c r="H5" s="21">
+      <c r="H5" s="6">
         <v>0.27300000000000002</v>
       </c>
-      <c r="I5" s="21">
+      <c r="I5" s="6">
         <v>0.255</v>
       </c>
-      <c r="J5" s="21">
+      <c r="J5" s="6">
         <v>8.5999999999999993E-2</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="21">
+      <c r="B6" s="6">
         <v>9.8000000000000004E-2</v>
       </c>
-      <c r="C6" s="21">
+      <c r="C6" s="6">
         <v>0.108</v>
       </c>
-      <c r="D6" s="21">
+      <c r="D6" s="6">
         <v>0.30399999999999999</v>
       </c>
-      <c r="E6" s="21">
+      <c r="E6" s="6">
         <v>0.29599999999999999</v>
       </c>
-      <c r="F6" s="21">
+      <c r="F6" s="6">
         <v>0.32500000000000001</v>
       </c>
-      <c r="G6" s="21">
+      <c r="G6" s="6">
         <v>0.24299999999999999</v>
       </c>
-      <c r="H6" s="21">
+      <c r="H6" s="6">
         <v>0.28799999999999998</v>
       </c>
-      <c r="I6" s="21">
+      <c r="I6" s="6">
         <v>0.251</v>
       </c>
-      <c r="J6" s="21">
+      <c r="J6" s="6">
         <v>0.09</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="21">
+      <c r="B7" s="6">
         <v>9.2999999999999999E-2</v>
       </c>
-      <c r="C7" s="21">
+      <c r="C7" s="6">
         <v>0.106</v>
       </c>
-      <c r="D7" s="21">
+      <c r="D7" s="6">
         <v>0.27100000000000002</v>
       </c>
-      <c r="E7" s="21">
+      <c r="E7" s="6">
         <v>0.28599999999999998</v>
       </c>
-      <c r="F7" s="21">
+      <c r="F7" s="6">
         <v>0.28499999999999998</v>
       </c>
-      <c r="G7" s="21">
+      <c r="G7" s="6">
         <v>0.192</v>
       </c>
-      <c r="H7" s="21">
+      <c r="H7" s="6">
         <v>0.23699999999999999</v>
       </c>
-      <c r="I7" s="21">
+      <c r="I7" s="6">
         <v>0.219</v>
       </c>
-      <c r="J7" s="21">
+      <c r="J7" s="6">
         <v>0.113</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="21">
+      <c r="B8" s="6">
         <v>9.6000000000000002E-2</v>
       </c>
-      <c r="C8" s="21">
+      <c r="C8" s="6">
         <v>9.9000000000000005E-2</v>
       </c>
-      <c r="D8" s="21">
+      <c r="D8" s="6">
         <v>0.255</v>
       </c>
-      <c r="E8" s="21">
+      <c r="E8" s="6">
         <v>0.309</v>
       </c>
-      <c r="F8" s="21">
+      <c r="F8" s="6">
         <v>0.27100000000000002</v>
       </c>
-      <c r="G8" s="21">
+      <c r="G8" s="6">
         <v>0.24199999999999999</v>
       </c>
-      <c r="H8" s="21">
+      <c r="H8" s="6">
         <v>0.192</v>
       </c>
-      <c r="I8" s="21">
+      <c r="I8" s="6">
         <v>0.187</v>
       </c>
-      <c r="J8" s="21">
+      <c r="J8" s="6">
         <v>8.7999999999999995E-2</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A9" s="9" t="s">
+      <c r="A9" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="21">
+      <c r="B9" s="6">
         <v>9.4E-2</v>
       </c>
-      <c r="C9" s="21">
+      <c r="C9" s="6">
         <v>9.7000000000000003E-2</v>
       </c>
-      <c r="D9" s="21">
+      <c r="D9" s="6">
         <v>0.19400000000000001</v>
       </c>
-      <c r="E9" s="21">
+      <c r="E9" s="6">
         <v>0.28799999999999998</v>
       </c>
-      <c r="F9" s="21">
+      <c r="F9" s="6">
         <v>0.26200000000000001</v>
       </c>
-      <c r="G9" s="21">
+      <c r="G9" s="6">
         <v>0.222</v>
       </c>
-      <c r="H9" s="21">
+      <c r="H9" s="6">
         <v>0.17100000000000001</v>
       </c>
-      <c r="I9" s="21">
+      <c r="I9" s="6">
         <v>0.157</v>
       </c>
-      <c r="J9" s="21">
+      <c r="J9" s="6">
         <v>0.1</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A10" s="9" t="s">
+      <c r="A10" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="21">
+      <c r="B10" s="6">
         <v>8.7999999999999995E-2</v>
       </c>
-      <c r="C10" s="21">
+      <c r="C10" s="6">
         <v>8.3000000000000004E-2</v>
       </c>
-      <c r="D10" s="21">
+      <c r="D10" s="6">
         <v>0.13600000000000001</v>
       </c>
-      <c r="E10" s="21">
+      <c r="E10" s="6">
         <v>0.251</v>
       </c>
-      <c r="F10" s="21">
+      <c r="F10" s="6">
         <v>0.23899999999999999</v>
       </c>
-      <c r="G10" s="21">
+      <c r="G10" s="6">
         <v>0.183</v>
       </c>
-      <c r="H10" s="21">
+      <c r="H10" s="6">
         <v>0.13900000000000001</v>
       </c>
-      <c r="I10" s="21">
+      <c r="I10" s="6">
         <v>0.127</v>
       </c>
-      <c r="J10" s="21">
+      <c r="J10" s="6">
         <v>8.2000000000000003E-2</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A11" s="9" t="s">
+      <c r="A11" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="21">
+      <c r="B11" s="6">
         <v>8.6999999999999994E-2</v>
       </c>
-      <c r="C11" s="21">
+      <c r="C11" s="6">
         <v>8.1000000000000003E-2</v>
       </c>
-      <c r="D11" s="21">
+      <c r="D11" s="6">
         <v>0.13500000000000001</v>
       </c>
-      <c r="E11" s="21">
+      <c r="E11" s="6">
         <v>0.21</v>
       </c>
-      <c r="F11" s="21">
+      <c r="F11" s="6">
         <v>0.19800000000000001</v>
       </c>
-      <c r="G11" s="21">
+      <c r="G11" s="6">
         <v>0.19</v>
       </c>
-      <c r="H11" s="21">
+      <c r="H11" s="6">
         <v>0.122</v>
       </c>
-      <c r="I11" s="21">
+      <c r="I11" s="6">
         <v>0.11</v>
       </c>
-      <c r="J11" s="21">
+      <c r="J11" s="6">
         <v>0.08</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B2:J8">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B2:J11">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -1913,7 +1888,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B2:J11">
+  <conditionalFormatting sqref="A2:A11">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>